<commit_message>
eval_arm_coco results: set1_night_aug all 3 splits (pycocotools)
</commit_message>
<xml_diff>
--- a/results/metrics_all_arms.xlsx
+++ b/results/metrics_all_arms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -432,6 +432,12 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,52 +473,82 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>mAP75</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>mAP50-95_bike</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>mAP50-95_bus</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>mAP50-95_car</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>mAP50-95_motor</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>mAP50-95_truck</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>mAP50_bike</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>mAP50_bus</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>mAP50_car</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>mAP50_motor</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>mAP50_truck</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>mAP75_bike</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>mAP75_bus</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>mAP75_car</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>mAP75_motor</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>mAP75_truck</t>
         </is>
       </c>
     </row>
@@ -543,34 +579,34 @@
       <c r="F2" t="n">
         <v>0.1821077785312609</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.05857757516387878</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>0.1813013955302692</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.3960492167078498</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>0.08079940273686101</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>0.1938113025174458</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>0.1342899123969109</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>0.2571064233153138</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>0.6850911920463809</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>0.1523301078095831</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>0.2976016399901913</v>
       </c>
     </row>
@@ -601,34 +637,34 @@
       <c r="F3" t="n">
         <v>0.1790582554831355</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>0.05916335017802149</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>0.1893399994639595</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>0.4090397248020623</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>0.04000926950609535</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>0.1977389334655389</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>0.1719540059705934</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>0.26030617074089</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>0.6778656118585755</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>0.08098228770287202</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>0.3018821362275799</v>
       </c>
     </row>
@@ -659,34 +695,34 @@
       <c r="F4" t="n">
         <v>0.1517324683726982</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>0.03837417500878087</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>0.1535417927400896</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>0.3502097366435195</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>0.01944927993295775</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>0.1970873575381435</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>0.1115250288351943</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>0.2213794032452082</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>0.6520888007203838</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>0.05782666011861951</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>0.293117965484832</v>
       </c>
     </row>
@@ -717,34 +753,34 @@
       <c r="F5" t="n">
         <v>0.1821077785312609</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>0.05857757516387878</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>0.1813013955302692</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>0.3960492167078498</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>0.08079940273686101</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>0.1938113025174458</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>0.1342899123969109</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>0.2571064233153138</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>0.6850911920463809</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>0.1523301078095831</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>0.2976016399901913</v>
       </c>
     </row>
@@ -775,34 +811,34 @@
       <c r="F6" t="n">
         <v>0.1790582554831355</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>0.05916335017802149</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>0.1893399994639595</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>0.4090397248020623</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>0.04000926950609535</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>0.1977389334655389</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>0.1719540059705934</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>0.26030617074089</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>0.6778656118585755</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>0.08098228770287202</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>0.3018821362275799</v>
       </c>
     </row>
@@ -833,34 +869,34 @@
       <c r="F7" t="n">
         <v>0.1517324683726982</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>0.03837417500878087</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>0.1535417927400896</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>0.3502097366435195</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>0.01944927993295775</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>0.1970873575381435</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>0.1115250288351943</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>0.2213794032452082</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>0.6520888007203838</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>0.05782666011861951</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>0.293117965484832</v>
       </c>
     </row>
@@ -891,34 +927,34 @@
       <c r="F8" t="n">
         <v>0.1821077785312609</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>0.05857757516387878</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>0.1813013955302692</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>0.3960492167078498</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>0.08079940273686101</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>0.1938113025174458</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>0.1342899123969109</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>0.2571064233153138</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>0.6850911920463809</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>0.1523301078095831</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>0.2976016399901913</v>
       </c>
     </row>
@@ -949,34 +985,34 @@
       <c r="F9" t="n">
         <v>0.1790582554831355</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>0.05916335017802149</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>0.1893399994639595</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>0.4090397248020623</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>0.04000926950609535</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>0.1977389334655389</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>0.1719540059705934</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>0.26030617074089</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>0.6778656118585755</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>0.08098228770287202</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>0.3018821362275799</v>
       </c>
     </row>
@@ -1007,34 +1043,34 @@
       <c r="F10" t="n">
         <v>0.1517324683726982</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>0.03837417500878087</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>0.1535417927400896</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>0.3502097366435195</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>0.01944927993295775</v>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>0.1970873575381435</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>0.1115250288351943</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>0.2213794032452082</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>0.6520888007203838</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>0.05782666011861951</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>0.293117965484832</v>
       </c>
     </row>
@@ -1065,34 +1101,34 @@
       <c r="F11" t="n">
         <v>0.1821077785312609</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>0.05857757516387878</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>0.1813013955302692</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>0.3960492167078498</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>0.08079940273686101</v>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>0.1938113025174458</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>0.1342899123969109</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>0.2571064233153138</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>0.6850911920463809</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>0.1523301078095831</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>0.2976016399901913</v>
       </c>
     </row>
@@ -1123,34 +1159,34 @@
       <c r="F12" t="n">
         <v>0.1790582554831355</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>0.05916335017802149</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>0.1893399994639595</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>0.4090397248020623</v>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>0.04000926950609535</v>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>0.1977389334655389</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>0.1719540059705934</v>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>0.26030617074089</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>0.6778656118585755</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>0.08098228770287202</v>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>0.3018821362275799</v>
       </c>
     </row>
@@ -1181,34 +1217,34 @@
       <c r="F13" t="n">
         <v>0.1694676058866271</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>0.05189771958791568</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>0.1375933791892869</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>0.4149946582734192</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>0.04768741669201867</v>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>0.1951648556904949</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>0.1375840949234592</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>0.1998616684221127</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>0.6864390943399843</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>0.1146779119947273</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>0.2937286372781098</v>
       </c>
     </row>
@@ -1239,34 +1275,34 @@
       <c r="F14" t="n">
         <v>0.1517324683726982</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>0.03837417500878087</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>0.1535417927400896</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>0.3502097366435195</v>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
         <v>0.01944927993295775</v>
       </c>
-      <c r="K14" t="n">
+      <c r="L14" t="n">
         <v>0.1970873575381435</v>
       </c>
-      <c r="L14" t="n">
+      <c r="M14" t="n">
         <v>0.1115250288351943</v>
       </c>
-      <c r="M14" t="n">
+      <c r="N14" t="n">
         <v>0.2213794032452082</v>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>0.6520888007203838</v>
       </c>
-      <c r="O14" t="n">
+      <c r="P14" t="n">
         <v>0.05782666011861951</v>
       </c>
-      <c r="P14" t="n">
+      <c r="Q14" t="n">
         <v>0.293117965484832</v>
       </c>
     </row>
@@ -1297,34 +1333,34 @@
       <c r="F15" t="n">
         <v>0.3871220486009554</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>0.2728993601128687</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>0.4723224486552465</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>0.4889988640701858</v>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
         <v>0.23753290754277</v>
       </c>
-      <c r="K15" t="n">
+      <c r="L15" t="n">
         <v>0.4638566626237067</v>
       </c>
-      <c r="L15" t="n">
+      <c r="M15" t="n">
         <v>0.5494994340203249</v>
       </c>
-      <c r="M15" t="n">
+      <c r="N15" t="n">
         <v>0.6192393725406993</v>
       </c>
-      <c r="N15" t="n">
+      <c r="O15" t="n">
         <v>0.7994316043357315</v>
       </c>
-      <c r="O15" t="n">
+      <c r="P15" t="n">
         <v>0.4777788533656264</v>
       </c>
-      <c r="P15" t="n">
+      <c r="Q15" t="n">
         <v>0.6383136990977132</v>
       </c>
     </row>
@@ -1355,34 +1391,34 @@
       <c r="F16" t="n">
         <v>0.3850966070676673</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>0.2504239395832958</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>0.553226848239898</v>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>0.5036871387366137</v>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>0.1226428674722721</v>
       </c>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>0.495502241306257</v>
       </c>
-      <c r="L16" t="n">
+      <c r="M16" t="n">
         <v>0.4906915445012149</v>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>0.6944839004141257</v>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>0.7967375435597949</v>
       </c>
-      <c r="O16" t="n">
+      <c r="P16" t="n">
         <v>0.2870432413723317</v>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>0.666356973738254</v>
       </c>
     </row>
@@ -1413,34 +1449,34 @@
       <c r="F17" t="n">
         <v>0.3655833267258713</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>0.1962456840831417</v>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
         <v>0.4565731490210802</v>
       </c>
-      <c r="I17" t="n">
+      <c r="J17" t="n">
         <v>0.5117632050880873</v>
       </c>
-      <c r="J17" t="n">
+      <c r="K17" t="n">
         <v>0.2035002850977668</v>
       </c>
-      <c r="K17" t="n">
+      <c r="L17" t="n">
         <v>0.4598343103392805</v>
       </c>
-      <c r="L17" t="n">
+      <c r="M17" t="n">
         <v>0.3970749033947613</v>
       </c>
-      <c r="M17" t="n">
+      <c r="N17" t="n">
         <v>0.6076061981997616</v>
       </c>
-      <c r="N17" t="n">
+      <c r="O17" t="n">
         <v>0.8051554078219201</v>
       </c>
-      <c r="O17" t="n">
+      <c r="P17" t="n">
         <v>0.4136205807263094</v>
       </c>
-      <c r="P17" t="n">
+      <c r="Q17" t="n">
         <v>0.6280104086135064</v>
       </c>
     </row>
@@ -1471,34 +1507,34 @@
       <c r="F18" t="n">
         <v>0.3563184614055295</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>0.2510302057586446</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>0.4537793114805136</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>0.4397865159026869</v>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
         <v>0.1880405810859183</v>
       </c>
-      <c r="K18" t="n">
+      <c r="L18" t="n">
         <v>0.448955692799884</v>
       </c>
-      <c r="L18" t="n">
+      <c r="M18" t="n">
         <v>0.493751576980352</v>
       </c>
-      <c r="M18" t="n">
+      <c r="N18" t="n">
         <v>0.5836455844003839</v>
       </c>
-      <c r="N18" t="n">
+      <c r="O18" t="n">
         <v>0.768540287308475</v>
       </c>
-      <c r="O18" t="n">
+      <c r="P18" t="n">
         <v>0.4169054633858057</v>
       </c>
-      <c r="P18" t="n">
+      <c r="Q18" t="n">
         <v>0.6157790753592082</v>
       </c>
     </row>
@@ -1529,34 +1565,34 @@
       <c r="F19" t="n">
         <v>0.3850653434857499</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>0.2504183470634505</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>0.5532136407126016</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>0.5037057076205904</v>
       </c>
-      <c r="J19" t="n">
+      <c r="K19" t="n">
         <v>0.1226428674722721</v>
       </c>
-      <c r="K19" t="n">
+      <c r="L19" t="n">
         <v>0.4953461545598354</v>
       </c>
-      <c r="L19" t="n">
+      <c r="M19" t="n">
         <v>0.4906904970721018</v>
       </c>
-      <c r="M19" t="n">
+      <c r="N19" t="n">
         <v>0.6944561917883567</v>
       </c>
-      <c r="N19" t="n">
+      <c r="O19" t="n">
         <v>0.7967430467784407</v>
       </c>
-      <c r="O19" t="n">
+      <c r="P19" t="n">
         <v>0.2870432413723317</v>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>0.6663355979755337</v>
       </c>
     </row>
@@ -1587,34 +1623,34 @@
       <c r="F20" t="n">
         <v>0.3655785789273447</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>0.1962090286934781</v>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>0.456749738303713</v>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>0.5117466734544206</v>
       </c>
-      <c r="J20" t="n">
+      <c r="K20" t="n">
         <v>0.2033444095616081</v>
       </c>
-      <c r="K20" t="n">
+      <c r="L20" t="n">
         <v>0.4598430446235039</v>
       </c>
-      <c r="L20" t="n">
+      <c r="M20" t="n">
         <v>0.3970496195276192</v>
       </c>
-      <c r="M20" t="n">
+      <c r="N20" t="n">
         <v>0.6076298094323311</v>
       </c>
-      <c r="N20" t="n">
+      <c r="O20" t="n">
         <v>0.8051131404924865</v>
       </c>
-      <c r="O20" t="n">
+      <c r="P20" t="n">
         <v>0.4132723557799116</v>
       </c>
-      <c r="P20" t="n">
+      <c r="Q20" t="n">
         <v>0.6279971673666702</v>
       </c>
     </row>
@@ -1645,35 +1681,263 @@
       <c r="F21" t="n">
         <v>0.3562938482545149</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>0.2505552585749934</v>
       </c>
-      <c r="H21" t="n">
+      <c r="I21" t="n">
         <v>0.4538084388659521</v>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>0.4398132034146327</v>
       </c>
-      <c r="J21" t="n">
+      <c r="K21" t="n">
         <v>0.1882869318421512</v>
       </c>
-      <c r="K21" t="n">
+      <c r="L21" t="n">
         <v>0.4490054085748453</v>
       </c>
-      <c r="L21" t="n">
+      <c r="M21" t="n">
         <v>0.4895021114529651</v>
       </c>
-      <c r="M21" t="n">
+      <c r="N21" t="n">
         <v>0.5836987233597186</v>
       </c>
-      <c r="N21" t="n">
+      <c r="O21" t="n">
         <v>0.7686801473409888</v>
       </c>
-      <c r="O21" t="n">
+      <c r="P21" t="n">
         <v>0.4171125724879096</v>
       </c>
-      <c r="P21" t="n">
+      <c r="Q21" t="n">
         <v>0.6157502584833824</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-17T13:35:32.536079+00:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>val_dawndusk</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.5696099999999999</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.36801</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.3816</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.26408</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.50209</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.49457</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.12671</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.45258</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.51974</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.63143</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.79522</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.29349</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.60814</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.22918</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0.56167</v>
+      </c>
+      <c r="T22" t="n">
+        <v>0.50258</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0.11262</v>
+      </c>
+      <c r="V22" t="n">
+        <v>0.50192</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-17T13:35:32.536079+00:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>val_day</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.53571</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.34311</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.35241</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.19494</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.40561</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.5024999999999999</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.19064</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.42183</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.39562</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.52755</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.80101</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.37778</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.5766</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.17977</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0.44764</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0.50886</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0.16657</v>
+      </c>
+      <c r="V23" t="n">
+        <v>0.45921</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-17T13:35:32.536079+00:00</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>val_night</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.54259</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.33508</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.33839</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.25695</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.40418</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.43328</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.17956</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.40141</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.49232</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.51744</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.76758</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.38715</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.54843</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0.23554</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.4599</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0.41106</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0.13437</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0.45108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
convert existing UTC timestamps to Thai time (UTC+7)
Retroactively shifts every timestamp already in metrics_all_arms.csv|xlsx
(348 rows) and results/logs/*.log to the same +07:00 offset new rows use
going forward - same instant in time, just displayed consistently in Thai
local time everywhere instead of a UTC/Thai mix.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/metrics_all_arms.xlsx
+++ b/results/metrics_all_arms.xlsx
@@ -555,7 +555,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-16T08:58:04.926074+00:00</t>
+          <t>2026-08-16T15:58:04.926074+07:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -613,7 +613,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-16T08:58:04.926074+00:00</t>
+          <t>2026-08-16T15:58:04.926074+07:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -671,7 +671,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-16T08:58:04.926074+00:00</t>
+          <t>2026-08-16T15:58:04.926074+07:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -729,7 +729,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-16T10:08:10.325959+00:00</t>
+          <t>2026-08-16T17:08:10.325959+07:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -787,7 +787,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-16T10:08:10.325959+00:00</t>
+          <t>2026-08-16T17:08:10.325959+07:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -845,7 +845,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-16T10:08:10.325959+00:00</t>
+          <t>2026-08-16T17:08:10.325959+07:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -903,7 +903,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-16T10:31:31.244659+00:00</t>
+          <t>2026-08-16T17:31:31.244659+07:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -961,7 +961,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-16T10:31:31.244659+00:00</t>
+          <t>2026-08-16T17:31:31.244659+07:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1019,7 +1019,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-16T10:31:31.244659+00:00</t>
+          <t>2026-08-16T17:31:31.244659+07:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1077,7 +1077,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-16T11:06:41.674227+00:00</t>
+          <t>2026-08-16T18:06:41.674227+07:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1135,7 +1135,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-16T11:06:41.674227+00:00</t>
+          <t>2026-08-16T18:06:41.674227+07:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1193,7 +1193,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-16T11:06:41.674227+00:00</t>
+          <t>2026-08-16T18:06:41.674227+07:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1251,7 +1251,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-16T11:06:41.674227+00:00</t>
+          <t>2026-08-16T18:06:41.674227+07:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1309,7 +1309,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-16T23:02:43.149658+00:00</t>
+          <t>2026-08-17T06:02:43.149658+07:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-16T23:02:43.149658+00:00</t>
+          <t>2026-08-17T06:02:43.149658+07:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1425,7 +1425,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-16T23:02:43.149658+00:00</t>
+          <t>2026-08-17T06:02:43.149658+07:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1483,7 +1483,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-16T23:02:43.149658+00:00</t>
+          <t>2026-08-17T06:02:43.149658+07:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1541,7 +1541,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-17T09:01:57.206545+00:00</t>
+          <t>2026-08-17T16:01:57.206545+07:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1599,7 +1599,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-17T09:01:57.206545+00:00</t>
+          <t>2026-08-17T16:01:57.206545+07:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1657,7 +1657,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-17T09:01:57.206545+00:00</t>
+          <t>2026-08-17T16:01:57.206545+07:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1715,7 +1715,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-17T13:35:32.536079+00:00</t>
+          <t>2026-08-17T20:35:32.536079+07:00</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1791,7 +1791,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-17T13:35:32.536079+00:00</t>
+          <t>2026-08-17T20:35:32.536079+07:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1867,7 +1867,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-17T13:35:32.536079+00:00</t>
+          <t>2026-08-17T20:35:32.536079+07:00</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1943,7 +1943,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-17T13:50:43.613339+00:00</t>
+          <t>2026-08-17T20:50:43.613339+07:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2019,7 +2019,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-17T13:50:43.613339+00:00</t>
+          <t>2026-08-17T20:50:43.613339+07:00</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2095,7 +2095,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-17T13:50:43.613339+00:00</t>
+          <t>2026-08-17T20:50:43.613339+07:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">

</xml_diff>